<commit_message>
dividing the question bank export .xlsx file to  one  sheet per question type
</commit_message>
<xml_diff>
--- a/Backend/assets/question_bank_export_template.xlsx
+++ b/Backend/assets/question_bank_export_template.xlsx
@@ -9,20 +9,30 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="21600" windowHeight="9600"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="21600" windowHeight="9600" activeTab="5"/>
   </bookViews>
   <sheets>
-    <sheet name="Question Bank" sheetId="1" r:id="rId1"/>
+    <sheet name="Multiple Choice" sheetId="1" r:id="rId1"/>
+    <sheet name="Multi Select" sheetId="2" r:id="rId2"/>
+    <sheet name="True False" sheetId="3" r:id="rId3"/>
+    <sheet name="Essay" sheetId="4" r:id="rId4"/>
+    <sheet name="Short Answer" sheetId="5" r:id="rId5"/>
+    <sheet name="Code" sheetId="6" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Question Bank'!$A$7:$M$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Code!$A$7:$I$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Essay!$A$7:$I$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Multi Select'!$A$7:$M$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Multiple Choice'!$A$7:$M$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Short Answer'!$A$7:$I$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'True False'!$A$7:$I$7</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="17">
   <si>
     <t>Course Title:</t>
   </si>
@@ -79,7 +89,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -88,20 +98,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="9"/>
-      <color rgb="FFBFBFBF"/>
-      <name val="Arial"/>
-    </font>
-    <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF1F3864"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -125,7 +124,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -148,33 +147,29 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="FFD9D9D9"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -194,42 +189,29 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>57151</xdr:colOff>
+      <xdr:colOff>57150</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>104775</xdr:rowOff>
+      <xdr:rowOff>95251</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>1279140</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="1250642" cy="1314450"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Picture 2"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
+        <xdr:cNvPr id="2" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="57151" y="104775"/>
-          <a:ext cx="1221989" cy="1285875"/>
+          <a:off x="57150" y="95251"/>
+          <a:ext cx="1250642" cy="1314450"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -237,7 +219,187 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1250642" cy="1314450"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="57150" y="95250"/>
+          <a:ext cx="1250642" cy="1314450"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1250642" cy="1314450"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="57150" y="95250"/>
+          <a:ext cx="1250642" cy="1314450"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1250642" cy="1314450"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="57150" y="95250"/>
+          <a:ext cx="1250642" cy="1314450"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1250642" cy="1314450"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="57150" y="95250"/>
+          <a:ext cx="1250642" cy="1314450"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="1250642" cy="1314450"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Image 1" descr="Picture"/>
+        <xdr:cNvPicPr/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="57150" y="95250"/>
+          <a:ext cx="1250642" cy="1314450"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -529,114 +691,679 @@
   <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="45" customWidth="1"/>
-    <col min="7" max="10" width="18" customWidth="1"/>
-    <col min="11" max="11" width="25" customWidth="1"/>
-    <col min="12" max="12" width="35" customWidth="1"/>
-    <col min="13" max="13" width="20" customWidth="1"/>
+    <col min="1" max="1" width="20" style="1" customWidth="1"/>
+    <col min="2" max="2" width="30" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12" style="1" customWidth="1"/>
+    <col min="6" max="6" width="45" style="1" customWidth="1"/>
+    <col min="7" max="10" width="18" style="1" customWidth="1"/>
+    <col min="11" max="11" width="25" style="1" customWidth="1"/>
+    <col min="12" max="12" width="35" style="1" customWidth="1"/>
+    <col min="13" max="13" width="20" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="6"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="6"/>
+      <c r="A1" s="6"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="8"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="8"/>
     </row>
     <row r="2" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="3"/>
-      <c r="B2" s="4" t="s">
+      <c r="A2" s="6"/>
+      <c r="B2" s="5" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="6"/>
-      <c r="F2" s="4" t="s">
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="2" t="s">
         <v>1</v>
       </c>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
     </row>
     <row r="3" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="6"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="6"/>
+      <c r="A3" s="6"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="8"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="8"/>
     </row>
     <row r="4" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="3"/>
-      <c r="B4" s="4" t="s">
+      <c r="A4" s="6"/>
+      <c r="B4" s="5" t="s">
         <v>2</v>
       </c>
       <c r="C4" s="6"/>
-      <c r="F4" s="4" t="s">
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
     </row>
     <row r="5" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
+      <c r="A5" s="6"/>
     </row>
     <row r="6" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3"/>
+      <c r="A6" s="6"/>
     </row>
     <row r="7" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F7" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="G7" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="H7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="I7" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="J7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="K7" s="1" t="s">
+      <c r="K7" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="L7" s="1" t="s">
+      <c r="L7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="M7" s="1" t="s">
+      <c r="M7" s="3" t="s">
         <v>16</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A7:M7"/>
-  <mergeCells count="9">
+  <mergeCells count="7">
+    <mergeCell ref="B2:C2"/>
     <mergeCell ref="A1:A6"/>
-    <mergeCell ref="F2"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="G1:H1"/>
     <mergeCell ref="B4:C4"/>
-    <mergeCell ref="F4"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D3:E3"/>
-    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="G4:H4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20" style="1" customWidth="1"/>
+    <col min="2" max="2" width="30" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12" style="1" customWidth="1"/>
+    <col min="6" max="6" width="45" style="1" customWidth="1"/>
+    <col min="7" max="10" width="18" style="1" customWidth="1"/>
+    <col min="11" max="11" width="25" style="1" customWidth="1"/>
+    <col min="12" max="12" width="35" style="1" customWidth="1"/>
+    <col min="13" max="13" width="20" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="8"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="8"/>
+    </row>
+    <row r="2" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6"/>
+      <c r="B2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="6"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+    </row>
+    <row r="3" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="8"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="8"/>
+    </row>
+    <row r="4" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6"/>
+      <c r="B4" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="6"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+    </row>
+    <row r="5" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6"/>
+    </row>
+    <row r="6" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6"/>
+    </row>
+    <row r="7" spans="1:13" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:M7"/>
+  <mergeCells count="7">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="A1:A6"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="G4:H4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20" style="1" customWidth="1"/>
+    <col min="2" max="2" width="30" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12" style="1" customWidth="1"/>
+    <col min="6" max="6" width="45" style="1" customWidth="1"/>
+    <col min="7" max="7" width="25" style="1" customWidth="1"/>
+    <col min="8" max="8" width="35" style="1" customWidth="1"/>
+    <col min="9" max="9" width="20" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="8"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="8"/>
+    </row>
+    <row r="2" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6"/>
+      <c r="B2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="6"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+    </row>
+    <row r="3" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="8"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="8"/>
+    </row>
+    <row r="4" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6"/>
+      <c r="B4" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="6"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+    </row>
+    <row r="5" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6"/>
+    </row>
+    <row r="6" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6"/>
+    </row>
+    <row r="7" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:I7"/>
+  <mergeCells count="7">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="A1:A6"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="G4:H4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20" style="1" customWidth="1"/>
+    <col min="2" max="2" width="30" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12" style="1" customWidth="1"/>
+    <col min="6" max="6" width="45" style="1" customWidth="1"/>
+    <col min="7" max="7" width="25" style="1" customWidth="1"/>
+    <col min="8" max="8" width="35" style="1" customWidth="1"/>
+    <col min="9" max="9" width="20" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="8"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="8"/>
+    </row>
+    <row r="2" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6"/>
+      <c r="B2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="6"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+    </row>
+    <row r="3" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="8"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="8"/>
+    </row>
+    <row r="4" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6"/>
+      <c r="B4" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="6"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+    </row>
+    <row r="5" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6"/>
+    </row>
+    <row r="6" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6"/>
+    </row>
+    <row r="7" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:I7"/>
+  <mergeCells count="7">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="A1:A6"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="G4:H4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20" style="1" customWidth="1"/>
+    <col min="2" max="2" width="30" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12" style="1" customWidth="1"/>
+    <col min="6" max="6" width="45" style="1" customWidth="1"/>
+    <col min="7" max="7" width="25" style="1" customWidth="1"/>
+    <col min="8" max="8" width="35" style="1" customWidth="1"/>
+    <col min="9" max="9" width="20" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="8"/>
+    </row>
+    <row r="2" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6"/>
+      <c r="B2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="6"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+    </row>
+    <row r="3" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="8"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="8"/>
+    </row>
+    <row r="4" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6"/>
+      <c r="B4" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="6"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+    </row>
+    <row r="5" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+    </row>
+    <row r="6" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6"/>
+    </row>
+    <row r="7" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:I7"/>
+  <mergeCells count="7">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="A1:A6"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="G2:H2"/>
+    <mergeCell ref="G4:H4"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="20" style="1" customWidth="1"/>
+    <col min="2" max="2" width="30" style="1" customWidth="1"/>
+    <col min="3" max="3" width="12" style="1" customWidth="1"/>
+    <col min="4" max="4" width="16" style="1" customWidth="1"/>
+    <col min="5" max="5" width="12" style="1" customWidth="1"/>
+    <col min="6" max="6" width="45" style="1" customWidth="1"/>
+    <col min="7" max="7" width="25" style="1" customWidth="1"/>
+    <col min="8" max="8" width="35" style="1" customWidth="1"/>
+    <col min="9" max="9" width="20" style="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="8"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="8"/>
+    </row>
+    <row r="2" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6"/>
+      <c r="B2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="6"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+    </row>
+    <row r="3" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="8"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="8"/>
+    </row>
+    <row r="4" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6"/>
+      <c r="B4" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="6"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+    </row>
+    <row r="5" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6"/>
+    </row>
+    <row r="6" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6"/>
+    </row>
+    <row r="7" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A7:I7"/>
+  <mergeCells count="7">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="A1:A6"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="G2:H2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>